<commit_message>
etichetta di Milano (D-063)
milano: «Milanno» -> «Milano»; tolte le 6 forme attestate ormai uguali
all'etichetta. ABox 27.863 -> 27.857.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/References.xlsx
+++ b/data/source/xlsx/References.xlsx
@@ -6017,11 +6017,6 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>Milano</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6452,11 +6447,6 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>Milano</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8247,11 +8237,6 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="I214" t="inlineStr">
-        <is>
-          <t>Milano</t>
-        </is>
-      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -11247,11 +11232,6 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="I297" t="inlineStr">
-        <is>
-          <t>Milano</t>
-        </is>
-      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -15227,11 +15207,6 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="I408" t="inlineStr">
-        <is>
-          <t>Milano</t>
-        </is>
-      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -15265,11 +15240,6 @@
       <c r="H409" t="inlineStr">
         <is>
           <t>qp</t>
-        </is>
-      </c>
-      <c r="I409" t="inlineStr">
-        <is>
-          <t>Milano</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
punti aperti: Cassero e motivazioni in fase 3, tre occorrenze divise (D-074, D-075, D-076)
Cassero (ref_00404) rinviato alla fase 3 (manca l'entità di Sant'Ignazio):
IQ20 = 1 dichiarato. Divise in due occorrenze Sacro Cuore (QP 65), via
Merulana (QP 76), Santi Quattro (QP 105); estratti da verificare sul
volume (DC-23). StatusRationaleShape resta Warning (48, DC-22).
ABox 40.393 -> 40.472.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/References.xlsx
+++ b/data/source/xlsx/References.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I731"/>
+  <dimension ref="A1:I734"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5967,9 +5967,14 @@
       <c r="E152" t="n">
         <v>65</v>
       </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Prima menzione della pagina; la seconda e' un'occorrenza distinta (D-075). Estratto da verificare sul volume a stampa.</t>
+        </is>
+      </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Riferirono ad Ingravallo che la Gina, la pupilla, era tornata dar Sacro Core, in quer momento. Il giovedì rientrava all’una: per la colazione. [...] Sì, un po’ prima della Gina, che annava ar Sacro Core alle otto. Non volle sostare a quella vista: «Nun me riesce de guardalla.» Se fece er segno de la croce.</t>
+          <t>Riferirono ad Ingravallo che la Gina, la pupilla, era tornata dar Sacro Core, in quer momento.</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -6902,9 +6907,14 @@
       <c r="E178" t="n">
         <v>76</v>
       </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Prima menzione della pagina; la seconda e' un'occorrenza distinta (D-075). Estratto da verificare sul volume a stampa.</t>
+        </is>
+      </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>La mattina dopo i giornali diedero notizia del fatto. Era venerdì. Li cronisti e il telefono aveveno rotto l’anima tutta la sera: tanto a via Merulana che giù, a Sante Stefene. Sicché, la mattina, un subisso. «Orribile delitto a via Merulana,» gridavano li strilloni, co li pacchi fra li ginocchi de la gente: fino all’undici e tre quarti.</t>
+          <t>Li cronisti e il telefono aveveno rotto l’anima tutta la sera: tanto a via Merulana che giù, a Sante Stefene.</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -9242,9 +9252,14 @@
       <c r="E242" t="n">
         <v>105</v>
       </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Prima menzione della pagina; la seconda e' un'occorrenza distinta (D-075). Estratto da verificare sul volume a stampa.</t>
+        </is>
+      </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>E quella malinconia di Liliana. Quella specie di fissazione. E poi co li Santi Quattro là vicino. «Che Liliana, Madonna! guai a sentimme dì de portalla via da li Santi Quattro!»</t>
+          <t>E poi co li Santi Quattro là vicino.</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -26864,6 +26879,136 @@
       <c r="H731" t="inlineStr">
         <is>
           <t>qpa</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>ref_00731</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>sacro_cuore</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>capitolo_II</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>A 65</t>
+        </is>
+      </c>
+      <c r="E732" t="n">
+        <v>65</v>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>Seconda menzione della pagina, separata da ref_00151 (D-075). Estratto da verificare sul volume a stampa.</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>Sì, un po’ prima della Gina, che annava ar Sacro Core alle otto.</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>Sacro Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>ref_00732</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>via_merulana</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>capitolo_III</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>A 76</t>
+        </is>
+      </c>
+      <c r="E733" t="n">
+        <v>76</v>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>Seconda menzione della pagina, separata da ref_00177 (D-075). Estratto da verificare sul volume a stampa.</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>«Orribile delitto a via Merulana,» gridavano li strilloni, co li pacchi fra li ginocchi de la gente: fino all’undici e tre quarti.</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>qpa</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>ref_00733</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>santi_quattro_coronati</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>capitolo_IV</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>A 105</t>
+        </is>
+      </c>
+      <c r="E734" t="n">
+        <v>105</v>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>Seconda menzione della pagina, separata da ref_00241 (D-075). Estratto da verificare sul volume a stampa.</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>«Che Liliana, Madonna! guai a sentimme dì de portalla via da li Santi Quattro!»</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>Santi Quattro</t>
         </is>
       </c>
     </row>

</xml_diff>